<commit_message>
updated dataset for may
</commit_message>
<xml_diff>
--- a/facility_data_2026.xlsx
+++ b/facility_data_2026.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\AHF\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F4F48402-6BB8-419C-A4DB-A7B871AE678F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{458C4045-E0B6-4835-9D88-5E3C9B33A34D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="12645" yWindow="8025" windowWidth="13725" windowHeight="7215" xr2:uid="{FF4CAB09-7E04-4EC4-91FD-EE411994FF68}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{FF4CAB09-7E04-4EC4-91FD-EE411994FF68}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -801,8 +801,54 @@
       <c r="A6" t="s">
         <v>19</v>
       </c>
-      <c r="B6" s="3"/>
-      <c r="H6" s="3"/>
+      <c r="B6" s="3">
+        <v>1380</v>
+      </c>
+      <c r="C6">
+        <v>41</v>
+      </c>
+      <c r="D6">
+        <v>384</v>
+      </c>
+      <c r="E6">
+        <v>166</v>
+      </c>
+      <c r="F6">
+        <v>218</v>
+      </c>
+      <c r="G6">
+        <v>37</v>
+      </c>
+      <c r="H6" s="3">
+        <v>18576</v>
+      </c>
+      <c r="I6">
+        <v>39</v>
+      </c>
+      <c r="J6">
+        <v>22</v>
+      </c>
+      <c r="K6">
+        <v>32</v>
+      </c>
+      <c r="L6">
+        <v>24</v>
+      </c>
+      <c r="M6">
+        <v>18</v>
+      </c>
+      <c r="N6">
+        <v>2</v>
+      </c>
+      <c r="O6">
+        <v>356</v>
+      </c>
+      <c r="P6" s="2">
+        <v>0.91100000000000003</v>
+      </c>
+      <c r="Q6" s="2">
+        <v>0.95599999999999996</v>
+      </c>
     </row>
     <row r="7" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A7" t="s">

</xml_diff>